<commit_message>
fix: Add comma separator in list of strings
This resolves a missing separator present since commit

c44a15c ("Baseline from Hans dd 20240424.", 2024-04-29)

This issue appeared through reformatting of the source code, as the
concatenation of both strings (now happening on a single line) triggered
another linter/formatter warning.
</commit_message>
<xml_diff>
--- a/tests/eindhoven-500/reference/resultaten/werk/concurrentie/arbeidsplaatsen/restdag/Ontpl_conc_hoog.xlsx
+++ b/tests/eindhoven-500/reference/resultaten/werk/concurrentie/arbeidsplaatsen/restdag/Ontpl_conc_hoog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Zone</t>
   </si>
@@ -28,7 +28,10 @@
     <t>OV</t>
   </si>
   <si>
-    <t>Auto-FietsOV_Fiets</t>
+    <t>Auto-Fiets</t>
+  </si>
+  <si>
+    <t>OV_Fiets</t>
   </si>
   <si>
     <t>Auto_OV</t>
@@ -391,6 +394,9 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2">

</xml_diff>